<commit_message>
updated excel file sheet
</commit_message>
<xml_diff>
--- a/CAP766(PYTHON).xlsx
+++ b/CAP766(PYTHON).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\asus\Desktop\776\CAP776-GROUP-I-\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66FFF41E-B02C-4CEA-932B-024AEF7A043A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{714B8119-0BD3-415D-A4B0-C9846C65E92E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="82">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -269,6 +269,9 @@
   </si>
   <si>
     <t>Prep for CA TEST.</t>
+  </si>
+  <si>
+    <t>completed my First CA test in networking.</t>
   </si>
 </sst>
 </file>
@@ -2245,27 +2248,51 @@
         <v>80</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A32" s="13"/>
-      <c r="B32" s="14"/>
-      <c r="C32" s="14"/>
-      <c r="D32" s="14"/>
-      <c r="E32" s="14"/>
-      <c r="F32" s="14"/>
-      <c r="G32" s="14"/>
-      <c r="H32" s="14"/>
-      <c r="I32" s="15" t="str">
+    <row r="32" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A32" s="13">
+        <v>46272</v>
+      </c>
+      <c r="B32" s="14">
+        <v>360</v>
+      </c>
+      <c r="C32" s="14">
+        <v>40</v>
+      </c>
+      <c r="D32" s="14">
+        <v>120</v>
+      </c>
+      <c r="E32" s="14">
+        <v>0</v>
+      </c>
+      <c r="F32" s="14">
+        <v>150</v>
+      </c>
+      <c r="G32" s="14">
+        <v>3</v>
+      </c>
+      <c r="H32" s="14">
+        <v>180</v>
+      </c>
+      <c r="I32" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J32" s="15" t="str">
+        <v>850</v>
+      </c>
+      <c r="J32" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K32" s="16"/>
-      <c r="L32" s="16"/>
-      <c r="M32" s="16"/>
-      <c r="N32" s="17"/>
+        <v>590</v>
+      </c>
+      <c r="K32" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L32" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="M32" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N32" s="17" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A33" s="13"/>

</xml_diff>